<commit_message>
regionalized land use and fertilizer use modules
</commit_message>
<xml_diff>
--- a/Regionalied FeliX/Model Files/Reg_InitialValues.xlsx
+++ b/Regionalied FeliX/Model Files/Reg_InitialValues.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iiasahub-my.sharepoint.com/personal/yequanliang_iiasa_ac_at/Documents/research_iiasa/Felix-Model/version_oct_2023/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://iiasahub-my.sharepoint.com/personal/yequanliang_iiasa_ac_at/Documents/research_iiasa/Felix-Model/Regionalied FeliX/Model Files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="405" documentId="13_ncr:1_{BC87DD94-8A18-4A38-BD52-67B37BD28289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1251FF2B-DB05-40CD-B009-4768F221375C}"/>
+  <xr:revisionPtr revIDLastSave="411" documentId="13_ncr:1_{BC87DD94-8A18-4A38-BD52-67B37BD28289}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{84931982-18AA-4C02-A06E-A6A93D4B203D}"/>
   <bookViews>
-    <workbookView xWindow="25974" yWindow="-109" windowWidth="26301" windowHeight="14169" tabRatio="695" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="22932" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="695" firstSheet="6" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stocks" sheetId="1" r:id="rId1"/>
@@ -5158,15 +5158,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I91"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="49.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="11.625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="44.625" style="42" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.6640625" style="42" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7">
@@ -6480,7 +6480,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="14.95" customHeight="1">
+    <row r="58" spans="1:9" ht="15" customHeight="1">
       <c r="A58" s="41" t="s">
         <v>57</v>
       </c>
@@ -7284,15 +7284,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4AFB4B9F-BCD1-40DF-A2BC-2B5CAD943BB0}">
   <dimension ref="A1:I96"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="49.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="37.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="49.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="37.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="9" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="9" customWidth="1"/>
-    <col min="6" max="6" width="11.625" style="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="57.875" style="42" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="57.88671875" style="42" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8">
@@ -8612,7 +8612,7 @@
         <v>269</v>
       </c>
     </row>
-    <row r="58" spans="1:9" ht="14.95" customHeight="1">
+    <row r="58" spans="1:9" ht="15" customHeight="1">
       <c r="A58" s="41" t="s">
         <v>57</v>
       </c>
@@ -9503,19 +9503,19 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AP88"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="14.875" customWidth="1"/>
+    <col min="1" max="1" width="14.88671875" customWidth="1"/>
     <col min="2" max="22" width="10" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="11" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="12.5" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="14.6640625" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="12.44140625" bestFit="1" customWidth="1"/>
     <col min="26" max="26" width="11" bestFit="1" customWidth="1"/>
     <col min="28" max="28" width="12" bestFit="1" customWidth="1"/>
     <col min="30" max="30" width="11" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="14.95" thickBot="1">
+    <row r="1" spans="1:32" ht="15" thickBot="1">
       <c r="A1" s="2">
         <v>1900</v>
       </c>
@@ -9736,7 +9736,7 @@
         <v>133000000</v>
       </c>
     </row>
-    <row r="4" spans="1:32" ht="14.95" thickBot="1">
+    <row r="4" spans="1:32" ht="15" thickBot="1">
       <c r="A4" s="5" t="s">
         <v>111</v>
       </c>
@@ -9996,7 +9996,7 @@
         <v>74000000</v>
       </c>
     </row>
-    <row r="7" spans="1:32" ht="14.95" thickBot="1">
+    <row r="7" spans="1:32" ht="15" thickBot="1">
       <c r="A7" s="6" t="s">
         <v>111</v>
       </c>
@@ -10225,7 +10225,7 @@
       </c>
       <c r="W9" s="10"/>
     </row>
-    <row r="10" spans="1:32" ht="14.95" thickBot="1">
+    <row r="10" spans="1:32" ht="15" thickBot="1">
       <c r="A10" s="6" t="s">
         <v>111</v>
       </c>
@@ -10431,7 +10431,7 @@
       </c>
       <c r="W12" s="10"/>
     </row>
-    <row r="13" spans="1:32" ht="14.95" thickBot="1">
+    <row r="13" spans="1:32" ht="15" thickBot="1">
       <c r="A13" s="6" t="s">
         <v>111</v>
       </c>
@@ -10636,7 +10636,7 @@
       </c>
       <c r="W15" s="10"/>
     </row>
-    <row r="16" spans="1:32" ht="14.95" thickBot="1">
+    <row r="16" spans="1:32" ht="15" thickBot="1">
       <c r="A16" s="6" t="s">
         <v>111</v>
       </c>
@@ -10841,7 +10841,7 @@
       </c>
       <c r="W18" s="10"/>
     </row>
-    <row r="19" spans="1:42" ht="14.95" thickBot="1">
+    <row r="19" spans="1:42" ht="15" thickBot="1">
       <c r="A19" s="6" t="s">
         <v>111</v>
       </c>
@@ -10954,7 +10954,7 @@
       <c r="U20" s="10"/>
       <c r="V20" s="10"/>
     </row>
-    <row r="21" spans="1:42" ht="19.7" thickBot="1">
+    <row r="21" spans="1:42" ht="18.600000000000001" thickBot="1">
       <c r="A21" s="33" t="s">
         <v>472</v>
       </c>
@@ -10980,7 +10980,7 @@
       <c r="U21" s="10"/>
       <c r="V21" s="10"/>
     </row>
-    <row r="22" spans="1:42" ht="14.95" thickBot="1">
+    <row r="22" spans="1:42" ht="15" thickBot="1">
       <c r="A22" s="2">
         <v>1950</v>
       </c>
@@ -11187,7 +11187,7 @@
       <c r="X24" s="10"/>
       <c r="Y24" s="10"/>
     </row>
-    <row r="25" spans="1:42" ht="14.95" thickBot="1">
+    <row r="25" spans="1:42" ht="15" thickBot="1">
       <c r="A25" s="6" t="s">
         <v>111</v>
       </c>
@@ -11395,7 +11395,7 @@
       <c r="AO27" s="83"/>
       <c r="AP27" s="83"/>
     </row>
-    <row r="28" spans="1:42" ht="14.95" thickBot="1">
+    <row r="28" spans="1:42" ht="15" thickBot="1">
       <c r="A28" s="6" t="s">
         <v>111</v>
       </c>
@@ -11604,7 +11604,7 @@
       <c r="AO30" s="83"/>
       <c r="AP30" s="83"/>
     </row>
-    <row r="31" spans="1:42" ht="14.95" thickBot="1">
+    <row r="31" spans="1:42" ht="15" thickBot="1">
       <c r="A31" s="6" t="s">
         <v>111</v>
       </c>
@@ -11813,7 +11813,7 @@
       <c r="AO33" s="83"/>
       <c r="AP33" s="83"/>
     </row>
-    <row r="34" spans="1:42" ht="14.95" thickBot="1">
+    <row r="34" spans="1:42" ht="15" thickBot="1">
       <c r="A34" s="6" t="s">
         <v>111</v>
       </c>
@@ -12022,7 +12022,7 @@
       <c r="AO36" s="83"/>
       <c r="AP36" s="83"/>
     </row>
-    <row r="37" spans="1:42" ht="14.95" thickBot="1">
+    <row r="37" spans="1:42" ht="15" thickBot="1">
       <c r="A37" s="6" t="s">
         <v>111</v>
       </c>
@@ -12140,7 +12140,7 @@
       <c r="V38" s="69"/>
       <c r="Y38" s="10"/>
     </row>
-    <row r="39" spans="1:42" ht="14.95" thickBot="1">
+    <row r="39" spans="1:42" ht="15" thickBot="1">
       <c r="A39" s="6" t="s">
         <v>110</v>
       </c>
@@ -12231,7 +12231,7 @@
       <c r="AO39" s="83"/>
       <c r="AP39" s="83"/>
     </row>
-    <row r="40" spans="1:42" ht="14.95" thickBot="1">
+    <row r="40" spans="1:42" ht="15" thickBot="1">
       <c r="A40" s="6" t="s">
         <v>111</v>
       </c>
@@ -12398,17 +12398,17 @@
       <c r="V43" s="10"/>
       <c r="Y43" s="84"/>
     </row>
-    <row r="44" spans="1:42" ht="16.3">
+    <row r="44" spans="1:42" ht="15.6">
       <c r="A44" s="39"/>
       <c r="Y44" s="84"/>
     </row>
-    <row r="45" spans="1:42" ht="19.7" thickBot="1">
+    <row r="45" spans="1:42" ht="18.600000000000001" thickBot="1">
       <c r="A45" s="33" t="s">
         <v>211</v>
       </c>
       <c r="Y45" s="84"/>
     </row>
-    <row r="46" spans="1:42" ht="14.95" thickBot="1">
+    <row r="46" spans="1:42" ht="15" thickBot="1">
       <c r="A46" s="2">
         <v>1900</v>
       </c>
@@ -12591,7 +12591,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="49" spans="1:22" ht="14.95" thickBot="1">
+    <row r="49" spans="1:22" ht="15" thickBot="1">
       <c r="A49" s="66" t="s">
         <v>111</v>
       </c>
@@ -12795,7 +12795,7 @@
         <v>322</v>
       </c>
     </row>
-    <row r="52" spans="1:22" ht="14.95" thickBot="1">
+    <row r="52" spans="1:22" ht="15" thickBot="1">
       <c r="A52" s="66" t="s">
         <v>111</v>
       </c>
@@ -12999,7 +12999,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="55" spans="1:22" ht="14.95" thickBot="1">
+    <row r="55" spans="1:22" ht="15" thickBot="1">
       <c r="A55" s="66" t="s">
         <v>111</v>
       </c>
@@ -13203,7 +13203,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="58" spans="1:22" ht="14.95" thickBot="1">
+    <row r="58" spans="1:22" ht="15" thickBot="1">
       <c r="A58" s="66" t="s">
         <v>111</v>
       </c>
@@ -13407,7 +13407,7 @@
         <v>1543</v>
       </c>
     </row>
-    <row r="61" spans="1:22" ht="14.95" thickBot="1">
+    <row r="61" spans="1:22" ht="15" thickBot="1">
       <c r="A61" s="66" t="s">
         <v>111</v>
       </c>
@@ -13611,7 +13611,7 @@
         <v>2446</v>
       </c>
     </row>
-    <row r="64" spans="1:22" ht="14.95" thickBot="1">
+    <row r="64" spans="1:22" ht="15" thickBot="1">
       <c r="A64" s="66" t="s">
         <v>111</v>
       </c>
@@ -13700,8 +13700,8 @@
         <v>6101</v>
       </c>
     </row>
-    <row r="66" spans="1:24" ht="14.95" thickBot="1"/>
-    <row r="67" spans="1:24" ht="14.95" thickBot="1">
+    <row r="66" spans="1:24" ht="15" thickBot="1"/>
+    <row r="67" spans="1:24" ht="15" thickBot="1">
       <c r="A67" s="2">
         <v>2000</v>
       </c>
@@ -13865,7 +13865,7 @@
       </c>
       <c r="X69" s="10"/>
     </row>
-    <row r="70" spans="1:24" ht="14.95" thickBot="1">
+    <row r="70" spans="1:24" ht="15" thickBot="1">
       <c r="A70" s="66" t="s">
         <v>111</v>
       </c>
@@ -14030,7 +14030,7 @@
       </c>
       <c r="X72" s="10"/>
     </row>
-    <row r="73" spans="1:24" ht="14.95" thickBot="1">
+    <row r="73" spans="1:24" ht="15" thickBot="1">
       <c r="A73" s="66" t="s">
         <v>111</v>
       </c>
@@ -14195,7 +14195,7 @@
       </c>
       <c r="X75" s="10"/>
     </row>
-    <row r="76" spans="1:24" ht="14.95" thickBot="1">
+    <row r="76" spans="1:24" ht="15" thickBot="1">
       <c r="A76" s="66" t="s">
         <v>111</v>
       </c>
@@ -14360,7 +14360,7 @@
       </c>
       <c r="X78" s="10"/>
     </row>
-    <row r="79" spans="1:24" ht="14.95" thickBot="1">
+    <row r="79" spans="1:24" ht="15" thickBot="1">
       <c r="A79" s="66" t="s">
         <v>111</v>
       </c>
@@ -14525,7 +14525,7 @@
       </c>
       <c r="X81" s="10"/>
     </row>
-    <row r="82" spans="1:24" ht="14.95" thickBot="1">
+    <row r="82" spans="1:24" ht="15" thickBot="1">
       <c r="A82" s="66" t="s">
         <v>111</v>
       </c>
@@ -14623,27 +14623,27 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:AO98"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.375" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="6" width="10" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="8" max="15" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="15" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="10" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="9.375" customWidth="1"/>
+    <col min="17" max="17" width="9.33203125" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="19" width="15" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="11.375" customWidth="1"/>
-    <col min="21" max="21" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.625" customWidth="1"/>
-    <col min="23" max="29" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="9.375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.5" customWidth="1"/>
-    <col min="40" max="40" width="11.5" customWidth="1"/>
+    <col min="20" max="20" width="11.33203125" customWidth="1"/>
+    <col min="21" max="21" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" customWidth="1"/>
+    <col min="23" max="29" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.44140625" customWidth="1"/>
+    <col min="40" max="40" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:41" ht="19.7" thickBot="1">
+    <row r="1" spans="1:41" ht="18.600000000000001" thickBot="1">
       <c r="A1" s="33" t="s">
         <v>112</v>
       </c>
@@ -14773,7 +14773,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="4" spans="1:41" ht="14.95" thickBot="1">
+    <row r="4" spans="1:41" ht="15" thickBot="1">
       <c r="A4" s="14" t="s">
         <v>111</v>
       </c>
@@ -14835,7 +14835,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="5" spans="1:41" ht="14.95" thickBot="1"/>
+    <row r="5" spans="1:41" ht="15" thickBot="1"/>
     <row r="6" spans="1:41">
       <c r="A6" s="2">
         <v>1960</v>
@@ -14960,7 +14960,7 @@
         <v>591390.375</v>
       </c>
     </row>
-    <row r="8" spans="1:41" ht="14.95" thickBot="1">
+    <row r="8" spans="1:41" ht="15" thickBot="1">
       <c r="A8" s="14" t="s">
         <v>111</v>
       </c>
@@ -15022,7 +15022,7 @@
         <v>406745.5</v>
       </c>
     </row>
-    <row r="9" spans="1:41" ht="14.95" thickBot="1"/>
+    <row r="9" spans="1:41" ht="15" thickBot="1"/>
     <row r="10" spans="1:41">
       <c r="A10" s="2">
         <v>2016</v>
@@ -15267,7 +15267,7 @@
         <v>30920</v>
       </c>
     </row>
-    <row r="12" spans="1:41" ht="14.95" thickBot="1">
+    <row r="12" spans="1:41" ht="15" thickBot="1">
       <c r="A12" s="14" t="s">
         <v>111</v>
       </c>
@@ -15389,7 +15389,7 @@
         <v>141850</v>
       </c>
     </row>
-    <row r="14" spans="1:41" ht="19.7" thickBot="1">
+    <row r="14" spans="1:41" ht="18.600000000000001" thickBot="1">
       <c r="A14" s="33" t="s">
         <v>114</v>
       </c>
@@ -15513,7 +15513,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="17" spans="1:40" ht="14.95" thickBot="1">
+    <row r="17" spans="1:40" ht="15" thickBot="1">
       <c r="A17" s="14" t="s">
         <v>111</v>
       </c>
@@ -15572,7 +15572,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="18" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="18" spans="1:40" ht="15" thickBot="1"/>
     <row r="19" spans="1:40">
       <c r="A19" s="2">
         <v>1960</v>
@@ -15691,7 +15691,7 @@
         <v>495679.0625</v>
       </c>
     </row>
-    <row r="21" spans="1:40" ht="14.95" thickBot="1">
+    <row r="21" spans="1:40" ht="15" thickBot="1">
       <c r="A21" s="14" t="s">
         <v>111</v>
       </c>
@@ -15750,7 +15750,7 @@
         <v>426500.21875</v>
       </c>
     </row>
-    <row r="22" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="22" spans="1:40" ht="15" thickBot="1"/>
     <row r="23" spans="1:40">
       <c r="A23" s="2">
         <v>2016</v>
@@ -15983,7 +15983,7 @@
         <v>27390</v>
       </c>
     </row>
-    <row r="25" spans="1:40" ht="14.95" thickBot="1">
+    <row r="25" spans="1:40" ht="15" thickBot="1">
       <c r="A25" s="14" t="s">
         <v>111</v>
       </c>
@@ -16099,7 +16099,7 @@
         <v>125540</v>
       </c>
     </row>
-    <row r="27" spans="1:40" ht="19.7" thickBot="1">
+    <row r="27" spans="1:40" ht="18.600000000000001" thickBot="1">
       <c r="A27" s="33" t="s">
         <v>115</v>
       </c>
@@ -16218,7 +16218,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="30" spans="1:40" ht="14.95" thickBot="1">
+    <row r="30" spans="1:40" ht="15" thickBot="1">
       <c r="A30" s="14" t="s">
         <v>111</v>
       </c>
@@ -16274,7 +16274,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="31" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="31" spans="1:40" ht="15" thickBot="1"/>
     <row r="32" spans="1:40">
       <c r="A32" s="2">
         <v>1960</v>
@@ -16388,7 +16388,7 @@
         <v>97609.96875</v>
       </c>
     </row>
-    <row r="34" spans="1:40" ht="14.95" thickBot="1">
+    <row r="34" spans="1:40" ht="15" thickBot="1">
       <c r="A34" s="14" t="s">
         <v>111</v>
       </c>
@@ -16444,7 +16444,7 @@
         <v>84032.796875</v>
       </c>
     </row>
-    <row r="35" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="35" spans="1:40" ht="15" thickBot="1"/>
     <row r="36" spans="1:40">
       <c r="A36" s="2">
         <v>2016</v>
@@ -16667,7 +16667,7 @@
         <v>9460</v>
       </c>
     </row>
-    <row r="38" spans="1:40" ht="14.95" thickBot="1">
+    <row r="38" spans="1:40" ht="15" thickBot="1">
       <c r="A38" s="14" t="s">
         <v>111</v>
       </c>
@@ -16777,7 +16777,7 @@
         <v>18130</v>
       </c>
     </row>
-    <row r="40" spans="1:40" ht="19.7" thickBot="1">
+    <row r="40" spans="1:40" ht="18.600000000000001" thickBot="1">
       <c r="A40" s="33" t="s">
         <v>212</v>
       </c>
@@ -16907,7 +16907,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="43" spans="1:40" ht="14.95" thickBot="1">
+    <row r="43" spans="1:40" ht="15" thickBot="1">
       <c r="A43" s="14" t="s">
         <v>111</v>
       </c>
@@ -16969,7 +16969,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="44" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="44" spans="1:40" ht="15" thickBot="1"/>
     <row r="45" spans="1:40">
       <c r="A45" s="2" t="s">
         <v>114</v>
@@ -17088,7 +17088,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="47" spans="1:40" ht="14.95" thickBot="1">
+    <row r="47" spans="1:40" ht="15" thickBot="1">
       <c r="A47" s="14" t="s">
         <v>111</v>
       </c>
@@ -17147,7 +17147,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="48" spans="1:40" ht="14.95" thickBot="1"/>
+    <row r="48" spans="1:40" ht="15" thickBot="1"/>
     <row r="49" spans="1:20">
       <c r="A49" s="2" t="s">
         <v>115</v>
@@ -17260,7 +17260,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="51" spans="1:20" ht="14.95" thickBot="1">
+    <row r="51" spans="1:20" ht="15" thickBot="1">
       <c r="A51" s="14" t="s">
         <v>111</v>
       </c>
@@ -17332,7 +17332,7 @@
         <v>0.33414637284721094</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="19.7" thickBot="1">
+    <row r="55" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A55" s="33" t="s">
         <v>213</v>
       </c>
@@ -17462,7 +17462,7 @@
         <v>49439.903539999999</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="14.95" thickBot="1">
+    <row r="58" spans="1:20" ht="15" thickBot="1">
       <c r="A58" s="14" t="s">
         <v>111</v>
       </c>
@@ -17524,7 +17524,7 @@
         <v>205910.63190000001</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="59" spans="1:20" ht="15" thickBot="1"/>
     <row r="60" spans="1:20">
       <c r="A60" s="2" t="s">
         <v>114</v>
@@ -17643,7 +17643,7 @@
         <v>32184.73475</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="14.95" thickBot="1">
+    <row r="62" spans="1:20" ht="15" thickBot="1">
       <c r="A62" s="14" t="s">
         <v>111</v>
       </c>
@@ -17702,7 +17702,7 @@
         <v>147647.965</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="63" spans="1:20" ht="15" thickBot="1"/>
     <row r="64" spans="1:20">
       <c r="A64" s="2" t="s">
         <v>115</v>
@@ -17815,7 +17815,7 @@
         <v>11521.985650000001</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="14.95" thickBot="1">
+    <row r="66" spans="1:20" ht="15" thickBot="1">
       <c r="A66" s="14" t="s">
         <v>111</v>
       </c>
@@ -17871,7 +17871,7 @@
         <v>22798.98849</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="19.7" thickBot="1">
+    <row r="70" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A70" s="33" t="s">
         <v>314</v>
       </c>
@@ -18001,7 +18001,7 @@
         <v>3850857</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="14.95" thickBot="1">
+    <row r="73" spans="1:20" ht="15" thickBot="1">
       <c r="A73" s="14" t="s">
         <v>111</v>
       </c>
@@ -18063,7 +18063,7 @@
         <v>2626778.25</v>
       </c>
     </row>
-    <row r="74" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="74" spans="1:20" ht="15" thickBot="1"/>
     <row r="75" spans="1:20">
       <c r="A75" s="2" t="s">
         <v>114</v>
@@ -18182,7 +18182,7 @@
         <v>3745399.75</v>
       </c>
     </row>
-    <row r="77" spans="1:20" ht="14.95" thickBot="1">
+    <row r="77" spans="1:20" ht="15" thickBot="1">
       <c r="A77" s="14" t="s">
         <v>111</v>
       </c>
@@ -18241,7 +18241,7 @@
         <v>2715952</v>
       </c>
     </row>
-    <row r="78" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="78" spans="1:20" ht="15" thickBot="1"/>
     <row r="79" spans="1:20">
       <c r="A79" s="2" t="s">
         <v>115</v>
@@ -18354,7 +18354,7 @@
         <v>768252.25</v>
       </c>
     </row>
-    <row r="81" spans="1:20" ht="14.95" thickBot="1">
+    <row r="81" spans="1:20" ht="15" thickBot="1">
       <c r="A81" s="14" t="s">
         <v>111</v>
       </c>
@@ -18566,7 +18566,7 @@
         <v>5.3802224226029455E-2</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="19.7" thickBot="1">
+    <row r="87" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A87" s="33" t="s">
         <v>357</v>
       </c>
@@ -18715,7 +18715,7 @@
         <v>86.878056940274845</v>
       </c>
     </row>
-    <row r="90" spans="1:20" ht="14.95" thickBot="1">
+    <row r="90" spans="1:20" ht="15" thickBot="1">
       <c r="A90" s="14" t="s">
         <v>111</v>
       </c>
@@ -18796,7 +18796,7 @@
         <v>59.812200739650756</v>
       </c>
     </row>
-    <row r="91" spans="1:20" ht="14.95" thickBot="1">
+    <row r="91" spans="1:20" ht="15" thickBot="1">
       <c r="A91" s="15"/>
     </row>
     <row r="92" spans="1:20">
@@ -18935,7 +18935,7 @@
         <v>73.512202026386404</v>
       </c>
     </row>
-    <row r="94" spans="1:20" ht="14.95" thickBot="1">
+    <row r="94" spans="1:20" ht="15" thickBot="1">
       <c r="A94" s="14" t="s">
         <v>111</v>
       </c>
@@ -19012,7 +19012,7 @@
         <v>63.487810840970077</v>
       </c>
     </row>
-    <row r="95" spans="1:20" ht="14.95" thickBot="1">
+    <row r="95" spans="1:20" ht="15" thickBot="1">
       <c r="A95" s="15"/>
     </row>
     <row r="96" spans="1:20">
@@ -19144,7 +19144,7 @@
         <v>14.702440405277281</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="14.95" thickBot="1">
+    <row r="98" spans="1:18" ht="15" thickBot="1">
       <c r="A98" s="14" t="s">
         <v>111</v>
       </c>
@@ -19228,21 +19228,21 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DC4DFFBB-89E7-48FA-BE1F-C6391D6C3ADE}">
   <dimension ref="A1:X235"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="9.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="17" width="12" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="20" width="12" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.625" customWidth="1"/>
-    <col min="23" max="29" width="9.625" bestFit="1" customWidth="1"/>
-    <col min="30" max="31" width="9.375" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="10.5" customWidth="1"/>
-    <col min="40" max="40" width="11.5" customWidth="1"/>
+    <col min="21" max="21" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.6640625" customWidth="1"/>
+    <col min="23" max="29" width="9.6640625" bestFit="1" customWidth="1"/>
+    <col min="30" max="31" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="10.44140625" customWidth="1"/>
+    <col min="40" max="40" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" ht="14.95" thickBot="1">
+    <row r="1" spans="1:24" ht="15" thickBot="1">
       <c r="A1" s="91">
         <v>1900</v>
       </c>
@@ -19431,7 +19431,7 @@
         <v>1.0804480345796483</v>
       </c>
     </row>
-    <row r="4" spans="1:24" ht="14.95" thickBot="1">
+    <row r="4" spans="1:24" ht="15" thickBot="1">
       <c r="A4" s="112"/>
       <c r="B4" s="14" t="s">
         <v>111</v>
@@ -19620,7 +19620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="14.95" thickBot="1">
+    <row r="7" spans="1:24" ht="15" thickBot="1">
       <c r="A7" s="112"/>
       <c r="B7" s="14" t="s">
         <v>111</v>
@@ -19809,7 +19809,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:24" ht="14.95" thickBot="1">
+    <row r="10" spans="1:24" ht="15" thickBot="1">
       <c r="A10" s="112"/>
       <c r="B10" s="15" t="s">
         <v>111</v>
@@ -19998,7 +19998,7 @@
         <v>171.11570889877223</v>
       </c>
     </row>
-    <row r="13" spans="1:24" ht="14.95" thickBot="1">
+    <row r="13" spans="1:24" ht="15" thickBot="1">
       <c r="A13" s="112"/>
       <c r="B13" s="15" t="s">
         <v>111</v>
@@ -20187,7 +20187,7 @@
         <v>119.51829418662345</v>
       </c>
     </row>
-    <row r="16" spans="1:24" ht="14.95" thickBot="1">
+    <row r="16" spans="1:24" ht="15" thickBot="1">
       <c r="A16" s="112"/>
       <c r="B16" s="14" t="s">
         <v>111</v>
@@ -20376,7 +20376,7 @@
         <v>298.20353600554779</v>
       </c>
     </row>
-    <row r="19" spans="1:21" ht="14.95" thickBot="1">
+    <row r="19" spans="1:21" ht="15" thickBot="1">
       <c r="A19" s="113"/>
       <c r="B19" s="14" t="s">
         <v>111</v>
@@ -20458,7 +20458,7 @@
         <v>894.61061948648398</v>
       </c>
     </row>
-    <row r="20" spans="1:21" ht="14.95" thickBot="1">
+    <row r="20" spans="1:21" ht="15" thickBot="1">
       <c r="A20" s="111" t="s">
         <v>432</v>
       </c>
@@ -20620,7 +20620,7 @@
         <v>149.10176800277389</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="14.95" thickBot="1">
+    <row r="23" spans="1:21" ht="15" thickBot="1">
       <c r="A23" s="112"/>
       <c r="B23" s="14" t="s">
         <v>111</v>
@@ -20800,7 +20800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:21" ht="14.95" thickBot="1">
+    <row r="26" spans="1:21" ht="15" thickBot="1">
       <c r="A26" s="112"/>
       <c r="B26" s="15" t="s">
         <v>111</v>
@@ -20980,7 +20980,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:21" ht="14.95" thickBot="1">
+    <row r="29" spans="1:21" ht="15" thickBot="1">
       <c r="A29" s="112"/>
       <c r="B29" s="14" t="s">
         <v>111</v>
@@ -21160,7 +21160,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:21" ht="14.95" thickBot="1">
+    <row r="32" spans="1:21" ht="15" thickBot="1">
       <c r="A32" s="112"/>
       <c r="B32" s="15" t="s">
         <v>111</v>
@@ -21340,7 +21340,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:20" ht="14.95" thickBot="1">
+    <row r="35" spans="1:20" ht="15" thickBot="1">
       <c r="A35" s="112"/>
       <c r="B35" s="14" t="s">
         <v>111</v>
@@ -21520,7 +21520,7 @@
         <v>149.10176800277389</v>
       </c>
     </row>
-    <row r="38" spans="1:20" ht="14.95" thickBot="1">
+    <row r="38" spans="1:20" ht="15" thickBot="1">
       <c r="A38" s="113"/>
       <c r="B38" s="14" t="s">
         <v>111</v>
@@ -21598,7 +21598,7 @@
         <v>447.30530974324199</v>
       </c>
     </row>
-    <row r="39" spans="1:20" ht="14.95" thickBot="1">
+    <row r="39" spans="1:20" ht="15" thickBot="1">
       <c r="A39" s="111" t="s">
         <v>433</v>
       </c>
@@ -21752,7 +21752,7 @@
         <v>59.759147093311725</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="14.95" thickBot="1">
+    <row r="42" spans="1:20" ht="15" thickBot="1">
       <c r="A42" s="112"/>
       <c r="B42" s="14" t="s">
         <v>111</v>
@@ -21923,7 +21923,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="14.95" thickBot="1">
+    <row r="45" spans="1:20" ht="15" thickBot="1">
       <c r="A45" s="112"/>
       <c r="B45" s="15" t="s">
         <v>111</v>
@@ -22094,7 +22094,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="14.95" thickBot="1">
+    <row r="48" spans="1:20" ht="15" thickBot="1">
       <c r="A48" s="112"/>
       <c r="B48" s="14" t="s">
         <v>111</v>
@@ -22265,7 +22265,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:22" ht="14.95" thickBot="1">
+    <row r="51" spans="1:22" ht="15" thickBot="1">
       <c r="A51" s="112"/>
       <c r="B51" s="15" t="s">
         <v>111</v>
@@ -22436,7 +22436,7 @@
         <v>59.759147093311725</v>
       </c>
     </row>
-    <row r="54" spans="1:22" ht="14.95" thickBot="1">
+    <row r="54" spans="1:22" ht="15" thickBot="1">
       <c r="A54" s="112"/>
       <c r="B54" s="14" t="s">
         <v>111</v>
@@ -22607,7 +22607,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:22" ht="14.95" thickBot="1">
+    <row r="57" spans="1:22" ht="15" thickBot="1">
       <c r="A57" s="113"/>
       <c r="B57" s="14" t="s">
         <v>111</v>
@@ -22681,12 +22681,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:22" ht="19.7" thickBot="1">
+    <row r="59" spans="1:22" ht="18.600000000000001" thickBot="1">
       <c r="A59" s="33" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="14.95" thickBot="1">
+    <row r="60" spans="1:22" ht="15" thickBot="1">
       <c r="A60" s="91">
         <v>1950</v>
       </c>
@@ -22861,7 +22861,7 @@
         <v>192318600</v>
       </c>
     </row>
-    <row r="63" spans="1:22" ht="14.95" thickBot="1">
+    <row r="63" spans="1:22" ht="15" thickBot="1">
       <c r="A63" s="112"/>
       <c r="B63" s="14" t="s">
         <v>111</v>
@@ -23043,7 +23043,7 @@
         <v>1.9027800743141848E-2</v>
       </c>
     </row>
-    <row r="66" spans="1:23" ht="14.95" thickBot="1">
+    <row r="66" spans="1:23" ht="15" thickBot="1">
       <c r="A66" s="112"/>
       <c r="B66" s="14" t="s">
         <v>111</v>
@@ -23196,7 +23196,7 @@
         <v>0.47824131415266125</v>
       </c>
     </row>
-    <row r="69" spans="1:23" ht="14.95" thickBot="1">
+    <row r="69" spans="1:23" ht="15" thickBot="1">
       <c r="A69" s="112"/>
       <c r="B69" s="15" t="s">
         <v>111</v>
@@ -23367,7 +23367,7 @@
         <v>0.1827805526870516</v>
       </c>
     </row>
-    <row r="72" spans="1:23" ht="14.95" thickBot="1">
+    <row r="72" spans="1:23" ht="15" thickBot="1">
       <c r="A72" s="112"/>
       <c r="B72" s="14" t="s">
         <v>111</v>
@@ -23520,7 +23520,7 @@
         <v>5.0094478641171475E-2</v>
       </c>
     </row>
-    <row r="75" spans="1:23" ht="14.95" thickBot="1">
+    <row r="75" spans="1:23" ht="15" thickBot="1">
       <c r="A75" s="112"/>
       <c r="B75" s="15" t="s">
         <v>111</v>
@@ -23691,7 +23691,7 @@
         <v>0.26985585377597382</v>
       </c>
     </row>
-    <row r="78" spans="1:23" ht="14.95" thickBot="1">
+    <row r="78" spans="1:23" ht="15" thickBot="1">
       <c r="A78" s="113"/>
       <c r="B78" s="14" t="s">
         <v>111</v>
@@ -23763,7 +23763,7 @@
         <v>0.3675276299366888</v>
       </c>
     </row>
-    <row r="79" spans="1:23" ht="14.95" thickBot="1">
+    <row r="79" spans="1:23" ht="15" thickBot="1">
       <c r="A79" s="111" t="s">
         <v>432</v>
       </c>
@@ -23925,7 +23925,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="82" spans="1:20" ht="14.95" thickBot="1">
+    <row r="82" spans="1:20" ht="15" thickBot="1">
       <c r="A82" s="112"/>
       <c r="B82" s="14" t="s">
         <v>111</v>
@@ -24087,7 +24087,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="85" spans="1:20" ht="14.95" thickBot="1">
+    <row r="85" spans="1:20" ht="15" thickBot="1">
       <c r="A85" s="112"/>
       <c r="B85" s="15" t="s">
         <v>111</v>
@@ -24231,7 +24231,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="88" spans="1:20" ht="14.95" thickBot="1">
+    <row r="88" spans="1:20" ht="15" thickBot="1">
       <c r="A88" s="112"/>
       <c r="B88" s="14" t="s">
         <v>111</v>
@@ -24375,7 +24375,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="91" spans="1:20" ht="14.95" thickBot="1">
+    <row r="91" spans="1:20" ht="15" thickBot="1">
       <c r="A91" s="112"/>
       <c r="B91" s="15" t="s">
         <v>111</v>
@@ -24519,7 +24519,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="94" spans="1:20" ht="14.95" thickBot="1">
+    <row r="94" spans="1:20" ht="15" thickBot="1">
       <c r="A94" s="112"/>
       <c r="B94" s="14" t="s">
         <v>111</v>
@@ -24663,7 +24663,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="97" spans="1:20" ht="14.95" thickBot="1">
+    <row r="97" spans="1:20" ht="15" thickBot="1">
       <c r="A97" s="113"/>
       <c r="B97" s="14" t="s">
         <v>111</v>
@@ -24723,7 +24723,7 @@
         <v>600</v>
       </c>
     </row>
-    <row r="98" spans="1:20" ht="14.95" thickBot="1">
+    <row r="98" spans="1:20" ht="15" thickBot="1">
       <c r="A98" s="111" t="s">
         <v>433</v>
       </c>
@@ -24877,7 +24877,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="101" spans="1:20" ht="14.95" thickBot="1">
+    <row r="101" spans="1:20" ht="15" thickBot="1">
       <c r="A101" s="115"/>
       <c r="B101" s="14" t="s">
         <v>111</v>
@@ -25031,7 +25031,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="104" spans="1:20" ht="14.95" thickBot="1">
+    <row r="104" spans="1:20" ht="15" thickBot="1">
       <c r="A104" s="112"/>
       <c r="B104" s="15" t="s">
         <v>111</v>
@@ -25168,7 +25168,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="107" spans="1:20" ht="14.95" thickBot="1">
+    <row r="107" spans="1:20" ht="15" thickBot="1">
       <c r="A107" s="112"/>
       <c r="B107" s="14" t="s">
         <v>111</v>
@@ -25305,7 +25305,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="110" spans="1:20" ht="14.95" thickBot="1">
+    <row r="110" spans="1:20" ht="15" thickBot="1">
       <c r="A110" s="112"/>
       <c r="B110" s="15" t="s">
         <v>111</v>
@@ -25442,7 +25442,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="113" spans="1:21" ht="14.95" thickBot="1">
+    <row r="113" spans="1:21" ht="15" thickBot="1">
       <c r="A113" s="112"/>
       <c r="B113" s="14" t="s">
         <v>111</v>
@@ -25579,7 +25579,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="116" spans="1:21" ht="14.95" thickBot="1">
+    <row r="116" spans="1:21" ht="15" thickBot="1">
       <c r="A116" s="113"/>
       <c r="B116" s="14" t="s">
         <v>111</v>
@@ -25636,13 +25636,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="119" spans="1:21" ht="19.7" thickBot="1">
+    <row r="119" spans="1:21" ht="18.600000000000001" thickBot="1">
       <c r="A119" s="33" t="s">
         <v>357</v>
       </c>
       <c r="B119" s="33"/>
     </row>
-    <row r="120" spans="1:21" ht="14.95" thickBot="1">
+    <row r="120" spans="1:21" ht="15" thickBot="1">
       <c r="A120" s="96">
         <v>1950</v>
       </c>
@@ -25814,7 +25814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="123" spans="1:21" ht="14.95" thickBot="1">
+    <row r="123" spans="1:21" ht="15" thickBot="1">
       <c r="A123" s="109"/>
       <c r="B123" s="100" t="s">
         <v>111</v>
@@ -26003,7 +26003,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="126" spans="1:21" ht="14.95" thickBot="1">
+    <row r="126" spans="1:21" ht="15" thickBot="1">
       <c r="A126" s="109"/>
       <c r="B126" s="99" t="s">
         <v>111</v>
@@ -26192,7 +26192,7 @@
         <v>184.88163136538168</v>
       </c>
     </row>
-    <row r="129" spans="1:21" ht="14.95" thickBot="1">
+    <row r="129" spans="1:21" ht="15" thickBot="1">
       <c r="A129" s="109"/>
       <c r="B129" s="99" t="s">
         <v>111</v>
@@ -26381,7 +26381,7 @@
         <v>129.1333060502495</v>
       </c>
     </row>
-    <row r="132" spans="1:21" ht="14.95" thickBot="1">
+    <row r="132" spans="1:21" ht="15" thickBot="1">
       <c r="A132" s="109"/>
       <c r="B132" s="100" t="s">
         <v>111</v>
@@ -26570,7 +26570,7 @@
         <v>322.19342438189551</v>
       </c>
     </row>
-    <row r="135" spans="1:21" ht="14.95" thickBot="1">
+    <row r="135" spans="1:21" ht="15" thickBot="1">
       <c r="A135" s="110"/>
       <c r="B135" s="100" t="s">
         <v>111</v>
@@ -26652,7 +26652,7 @@
         <v>966.58028553825329</v>
       </c>
     </row>
-    <row r="136" spans="1:21" ht="14.95" thickBot="1">
+    <row r="136" spans="1:21" ht="15" thickBot="1">
       <c r="A136" s="109" t="s">
         <v>432</v>
       </c>
@@ -26814,7 +26814,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="139" spans="1:21" ht="14.95" thickBot="1">
+    <row r="139" spans="1:21" ht="15" thickBot="1">
       <c r="A139" s="109"/>
       <c r="B139" s="99" t="s">
         <v>111</v>
@@ -26994,7 +26994,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="142" spans="1:21" ht="14.95" thickBot="1">
+    <row r="142" spans="1:21" ht="15" thickBot="1">
       <c r="A142" s="109"/>
       <c r="B142" s="100" t="s">
         <v>111</v>
@@ -27174,7 +27174,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="145" spans="1:20" ht="14.95" thickBot="1">
+    <row r="145" spans="1:20" ht="15" thickBot="1">
       <c r="A145" s="109"/>
       <c r="B145" s="99" t="s">
         <v>111</v>
@@ -27354,7 +27354,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="148" spans="1:20" ht="14.95" thickBot="1">
+    <row r="148" spans="1:20" ht="15" thickBot="1">
       <c r="A148" s="109"/>
       <c r="B148" s="100" t="s">
         <v>111</v>
@@ -27534,7 +27534,7 @@
         <v>161.09671219094776</v>
       </c>
     </row>
-    <row r="151" spans="1:20" ht="14.95" thickBot="1">
+    <row r="151" spans="1:20" ht="15" thickBot="1">
       <c r="A151" s="110"/>
       <c r="B151" s="100" t="s">
         <v>111</v>
@@ -27612,7 +27612,7 @@
         <v>483.29014276912665</v>
       </c>
     </row>
-    <row r="152" spans="1:20" ht="14.95" thickBot="1">
+    <row r="152" spans="1:20" ht="15" thickBot="1">
       <c r="A152" s="109" t="s">
         <v>433</v>
       </c>
@@ -27766,7 +27766,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="155" spans="1:20" ht="14.95" thickBot="1">
+    <row r="155" spans="1:20" ht="15" thickBot="1">
       <c r="A155" s="109"/>
       <c r="B155" s="99" t="s">
         <v>111</v>
@@ -27937,7 +27937,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="158" spans="1:20" ht="14.95" thickBot="1">
+    <row r="158" spans="1:20" ht="15" thickBot="1">
       <c r="A158" s="109"/>
       <c r="B158" s="100" t="s">
         <v>111</v>
@@ -28108,7 +28108,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="161" spans="1:21" ht="14.95" thickBot="1">
+    <row r="161" spans="1:21" ht="15" thickBot="1">
       <c r="A161" s="109"/>
       <c r="B161" s="99" t="s">
         <v>111</v>
@@ -28279,7 +28279,7 @@
         <v>64.566653025124751</v>
       </c>
     </row>
-    <row r="164" spans="1:21" ht="14.95" thickBot="1">
+    <row r="164" spans="1:21" ht="15" thickBot="1">
       <c r="A164" s="109"/>
       <c r="B164" s="100" t="s">
         <v>111</v>
@@ -28450,7 +28450,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="167" spans="1:21" ht="14.95" thickBot="1">
+    <row r="167" spans="1:21" ht="15" thickBot="1">
       <c r="A167" s="110"/>
       <c r="B167" s="100" t="s">
         <v>111</v>
@@ -28524,7 +28524,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="168" spans="1:21" ht="14.95" thickBot="1">
+    <row r="168" spans="1:21" ht="15" thickBot="1">
       <c r="A168" s="109" t="s">
         <v>431</v>
       </c>
@@ -28694,7 +28694,7 @@
         <v>636.20836179752666</v>
       </c>
     </row>
-    <row r="171" spans="1:21" ht="14.95" thickBot="1">
+    <row r="171" spans="1:21" ht="15" thickBot="1">
       <c r="A171" s="109"/>
       <c r="B171" s="100" t="s">
         <v>111</v>
@@ -28776,7 +28776,7 @@
         <v>1221.9074560048641</v>
       </c>
     </row>
-    <row r="172" spans="1:21" ht="14.95" thickBot="1">
+    <row r="172" spans="1:21" ht="15" thickBot="1">
       <c r="A172" s="109" t="s">
         <v>432</v>
       </c>
@@ -28938,7 +28938,7 @@
         <v>161.09671219094776</v>
       </c>
     </row>
-    <row r="175" spans="1:21" ht="14.95" thickBot="1">
+    <row r="175" spans="1:21" ht="15" thickBot="1">
       <c r="A175" s="109"/>
       <c r="B175" s="100" t="s">
         <v>111</v>
@@ -29016,7 +29016,7 @@
         <v>547.85679602405889</v>
       </c>
     </row>
-    <row r="176" spans="1:21" ht="14.95" thickBot="1">
+    <row r="176" spans="1:21" ht="15" thickBot="1">
       <c r="A176" s="109" t="s">
         <v>433</v>
       </c>
@@ -29170,7 +29170,7 @@
         <v>64.566653025124751</v>
       </c>
     </row>
-    <row r="179" spans="1:20" ht="14.95" thickBot="1">
+    <row r="179" spans="1:20" ht="15" thickBot="1">
       <c r="A179" s="109"/>
       <c r="B179" s="100" t="s">
         <v>111</v>
@@ -29244,7 +29244,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="190" spans="1:20" ht="19.7" thickBot="1">
+    <row r="190" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A190" s="33" t="s">
         <v>212</v>
       </c>
@@ -29374,7 +29374,7 @@
         <v>260</v>
       </c>
     </row>
-    <row r="193" spans="1:20" ht="14.95" thickBot="1">
+    <row r="193" spans="1:20" ht="15" thickBot="1">
       <c r="A193" s="14" t="s">
         <v>111</v>
       </c>
@@ -29436,7 +29436,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="194" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="194" spans="1:20" ht="15" thickBot="1"/>
     <row r="195" spans="1:20">
       <c r="A195" s="2" t="s">
         <v>114</v>
@@ -29555,7 +29555,7 @@
         <v>220</v>
       </c>
     </row>
-    <row r="197" spans="1:20" ht="14.95" thickBot="1">
+    <row r="197" spans="1:20" ht="15" thickBot="1">
       <c r="A197" s="14" t="s">
         <v>111</v>
       </c>
@@ -29614,7 +29614,7 @@
         <v>190</v>
       </c>
     </row>
-    <row r="198" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="198" spans="1:20" ht="15" thickBot="1"/>
     <row r="199" spans="1:20">
       <c r="A199" s="2" t="s">
         <v>115</v>
@@ -29727,7 +29727,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="201" spans="1:20" ht="14.95" thickBot="1">
+    <row r="201" spans="1:20" ht="15" thickBot="1">
       <c r="A201" s="14" t="s">
         <v>111</v>
       </c>
@@ -29799,7 +29799,7 @@
         <v>0.33414637284721094</v>
       </c>
     </row>
-    <row r="205" spans="1:20" ht="19.7" thickBot="1">
+    <row r="205" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A205" s="33" t="s">
         <v>213</v>
       </c>
@@ -29929,7 +29929,7 @@
         <v>49439.903539999999</v>
       </c>
     </row>
-    <row r="208" spans="1:20" ht="14.95" thickBot="1">
+    <row r="208" spans="1:20" ht="15" thickBot="1">
       <c r="A208" s="14" t="s">
         <v>111</v>
       </c>
@@ -29991,7 +29991,7 @@
         <v>205910.63190000001</v>
       </c>
     </row>
-    <row r="209" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="209" spans="1:20" ht="15" thickBot="1"/>
     <row r="210" spans="1:20">
       <c r="A210" s="2" t="s">
         <v>114</v>
@@ -30110,7 +30110,7 @@
         <v>32184.73475</v>
       </c>
     </row>
-    <row r="212" spans="1:20" ht="14.95" thickBot="1">
+    <row r="212" spans="1:20" ht="15" thickBot="1">
       <c r="A212" s="14" t="s">
         <v>111</v>
       </c>
@@ -30169,7 +30169,7 @@
         <v>147647.965</v>
       </c>
     </row>
-    <row r="213" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="213" spans="1:20" ht="15" thickBot="1"/>
     <row r="214" spans="1:20">
       <c r="A214" s="2" t="s">
         <v>115</v>
@@ -30282,7 +30282,7 @@
         <v>11521.985650000001</v>
       </c>
     </row>
-    <row r="216" spans="1:20" ht="14.95" thickBot="1">
+    <row r="216" spans="1:20" ht="15" thickBot="1">
       <c r="A216" s="14" t="s">
         <v>111</v>
       </c>
@@ -30338,7 +30338,7 @@
         <v>22798.98849</v>
       </c>
     </row>
-    <row r="220" spans="1:20" ht="19.7" thickBot="1">
+    <row r="220" spans="1:20" ht="18.600000000000001" thickBot="1">
       <c r="A220" s="33" t="s">
         <v>314</v>
       </c>
@@ -30468,7 +30468,7 @@
         <v>3850857</v>
       </c>
     </row>
-    <row r="223" spans="1:20" ht="14.95" thickBot="1">
+    <row r="223" spans="1:20" ht="15" thickBot="1">
       <c r="A223" s="14" t="s">
         <v>111</v>
       </c>
@@ -30530,7 +30530,7 @@
         <v>2626778.25</v>
       </c>
     </row>
-    <row r="224" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="224" spans="1:20" ht="15" thickBot="1"/>
     <row r="225" spans="1:20">
       <c r="A225" s="2" t="s">
         <v>114</v>
@@ -30649,7 +30649,7 @@
         <v>3745399.75</v>
       </c>
     </row>
-    <row r="227" spans="1:20" ht="14.95" thickBot="1">
+    <row r="227" spans="1:20" ht="15" thickBot="1">
       <c r="A227" s="14" t="s">
         <v>111</v>
       </c>
@@ -30708,7 +30708,7 @@
         <v>2715952</v>
       </c>
     </row>
-    <row r="228" spans="1:20" ht="14.95" thickBot="1"/>
+    <row r="228" spans="1:20" ht="15" thickBot="1"/>
     <row r="229" spans="1:20">
       <c r="A229" s="2" t="s">
         <v>115</v>
@@ -30821,7 +30821,7 @@
         <v>768252.25</v>
       </c>
     </row>
-    <row r="231" spans="1:20" ht="14.95" thickBot="1">
+    <row r="231" spans="1:20" ht="15" thickBot="1">
       <c r="A231" s="14" t="s">
         <v>111</v>
       </c>
@@ -31058,16 +31058,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:AL276"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="13.5" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="14.375" customWidth="1"/>
-    <col min="37" max="37" width="9.625" customWidth="1"/>
-    <col min="39" max="39" width="15.375" customWidth="1"/>
-    <col min="40" max="40" width="17.625" customWidth="1"/>
+    <col min="1" max="1" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="14.33203125" customWidth="1"/>
+    <col min="37" max="37" width="9.6640625" customWidth="1"/>
+    <col min="39" max="39" width="15.33203125" customWidth="1"/>
+    <col min="40" max="40" width="17.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" ht="19.05">
+    <row r="1" spans="1:38" ht="18">
       <c r="A1" s="116">
         <v>1900</v>
       </c>
@@ -31111,7 +31111,7 @@
       <c r="AK1" s="116"/>
       <c r="AL1" s="116"/>
     </row>
-    <row r="2" spans="1:38" ht="19.7" thickBot="1">
+    <row r="2" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A2" s="17" t="s">
         <v>418</v>
       </c>
@@ -31215,7 +31215,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="3" spans="1:38" ht="14.95" thickBot="1">
+    <row r="3" spans="1:38" ht="15" thickBot="1">
       <c r="B3" t="s">
         <v>121</v>
       </c>
@@ -33020,7 +33020,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="25" spans="1:38" ht="19.7" thickBot="1">
+    <row r="25" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A25" s="17" t="s">
         <v>419</v>
       </c>
@@ -33121,7 +33121,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="26" spans="1:38" ht="14.95" thickBot="1">
+    <row r="26" spans="1:38" ht="15" thickBot="1">
       <c r="B26" t="s">
         <v>121</v>
       </c>
@@ -34926,7 +34926,7 @@
         <v>93754.1640625</v>
       </c>
     </row>
-    <row r="48" spans="1:38" ht="19.7" thickBot="1">
+    <row r="48" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A48" s="17" t="s">
         <v>420</v>
       </c>
@@ -35030,7 +35030,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="49" spans="2:38" ht="14.95" thickBot="1">
+    <row r="49" spans="2:38" ht="15" thickBot="1">
       <c r="B49" t="s">
         <v>121</v>
       </c>
@@ -36985,7 +36985,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="71" spans="1:38" ht="19.7" thickBot="1">
+    <row r="71" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A71" s="17" t="s">
         <v>421</v>
       </c>
@@ -37086,7 +37086,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="72" spans="1:38" ht="14.95" thickBot="1">
+    <row r="72" spans="1:38" ht="15" thickBot="1">
       <c r="B72" t="s">
         <v>121</v>
       </c>
@@ -39041,7 +39041,7 @@
         <v>93754.1640625</v>
       </c>
     </row>
-    <row r="94" spans="1:38" ht="19.7" thickBot="1">
+    <row r="94" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A94" s="17" t="s">
         <v>422</v>
       </c>
@@ -39145,7 +39145,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="95" spans="1:38" ht="14.95" thickBot="1">
+    <row r="95" spans="1:38" ht="15" thickBot="1">
       <c r="B95" t="s">
         <v>121</v>
       </c>
@@ -40950,7 +40950,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="117" spans="1:38" ht="19.7" thickBot="1">
+    <row r="117" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A117" s="17" t="s">
         <v>423</v>
       </c>
@@ -41051,7 +41051,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="118" spans="1:38" ht="14.95" thickBot="1">
+    <row r="118" spans="1:38" ht="15" thickBot="1">
       <c r="B118" t="s">
         <v>121</v>
       </c>
@@ -42856,7 +42856,7 @@
         <v>93754.1640625</v>
       </c>
     </row>
-    <row r="140" spans="1:38" ht="19.7" thickBot="1">
+    <row r="140" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A140" s="17" t="s">
         <v>424</v>
       </c>
@@ -42960,7 +42960,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="141" spans="1:38" ht="14.95" thickBot="1">
+    <row r="141" spans="1:38" ht="15" thickBot="1">
       <c r="B141" t="s">
         <v>121</v>
       </c>
@@ -44765,7 +44765,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="163" spans="1:38" ht="19.7" thickBot="1">
+    <row r="163" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A163" s="17" t="s">
         <v>425</v>
       </c>
@@ -44866,7 +44866,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="164" spans="1:38" ht="14.95" thickBot="1">
+    <row r="164" spans="1:38" ht="15" thickBot="1">
       <c r="B164" t="s">
         <v>121</v>
       </c>
@@ -46671,7 +46671,7 @@
         <v>93754.1640625</v>
       </c>
     </row>
-    <row r="186" spans="1:38" ht="19.7" thickBot="1">
+    <row r="186" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A186" s="17" t="s">
         <v>426</v>
       </c>
@@ -46775,7 +46775,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="187" spans="1:38" ht="14.95" thickBot="1">
+    <row r="187" spans="1:38" ht="15" thickBot="1">
       <c r="B187" t="s">
         <v>121</v>
       </c>
@@ -48580,7 +48580,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="209" spans="1:38" ht="19.7" thickBot="1">
+    <row r="209" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A209" s="17" t="s">
         <v>427</v>
       </c>
@@ -48681,7 +48681,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="210" spans="1:38" ht="14.95" thickBot="1">
+    <row r="210" spans="1:38" ht="15" thickBot="1">
       <c r="B210" t="s">
         <v>121</v>
       </c>
@@ -50486,7 +50486,7 @@
         <v>93754.1640625</v>
       </c>
     </row>
-    <row r="232" spans="1:38" ht="19.7" thickBot="1">
+    <row r="232" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A232" s="17" t="s">
         <v>428</v>
       </c>
@@ -50590,7 +50590,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="233" spans="1:38" ht="14.95" thickBot="1">
+    <row r="233" spans="1:38" ht="15" thickBot="1">
       <c r="B233" t="s">
         <v>121</v>
       </c>
@@ -52395,7 +52395,7 @@
         <v>469095.03125</v>
       </c>
     </row>
-    <row r="255" spans="1:38" ht="19.7" thickBot="1">
+    <row r="255" spans="1:38" ht="18.600000000000001" thickBot="1">
       <c r="A255" s="17" t="s">
         <v>429</v>
       </c>
@@ -52496,7 +52496,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="256" spans="1:38" ht="14.95" thickBot="1">
+    <row r="256" spans="1:38" ht="15" thickBot="1">
       <c r="B256" t="s">
         <v>121</v>
       </c>
@@ -54316,7 +54316,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:V13"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:22">
       <c r="A1" t="s">
@@ -55206,13 +55206,13 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89F7AE5B-F9A7-4EA8-8D55-61A6797D1EA8}">
   <dimension ref="A1:V84"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="2" max="17" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="10.625" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="10.375" bestFit="1" customWidth="1"/>
-    <col min="20" max="21" width="10.625" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="10.375" bestFit="1" customWidth="1"/>
+    <col min="2" max="17" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="20" max="21" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="10.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:22">
@@ -55919,7 +55919,7 @@
         <v>3.8188840000000002</v>
       </c>
     </row>
-    <row r="12" spans="1:22" ht="14.95" thickBot="1"/>
+    <row r="12" spans="1:22" ht="15" thickBot="1"/>
     <row r="13" spans="1:22">
       <c r="A13" s="72" t="s">
         <v>404</v>
@@ -56624,7 +56624,7 @@
         <v>59.644039999999997</v>
       </c>
     </row>
-    <row r="24" spans="1:22" ht="14.95" thickBot="1"/>
+    <row r="24" spans="1:22" ht="15" thickBot="1"/>
     <row r="25" spans="1:22">
       <c r="A25" s="72" t="s">
         <v>405</v>
@@ -57329,7 +57329,7 @@
         <v>2.208701</v>
       </c>
     </row>
-    <row r="36" spans="1:22" ht="14.95" thickBot="1"/>
+    <row r="36" spans="1:22" ht="15" thickBot="1"/>
     <row r="37" spans="1:22">
       <c r="A37" s="72" t="s">
         <v>406</v>
@@ -58034,7 +58034,7 @@
         <v>-7.9391400000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:22" ht="14.95" thickBot="1"/>
+    <row r="48" spans="1:22" ht="15" thickBot="1"/>
     <row r="49" spans="1:22">
       <c r="A49" s="72" t="s">
         <v>407</v>
@@ -58739,7 +58739,7 @@
         <v>3.9565169999999998</v>
       </c>
     </row>
-    <row r="60" spans="1:22" ht="14.95" thickBot="1"/>
+    <row r="60" spans="1:22" ht="15" thickBot="1"/>
     <row r="61" spans="1:22">
       <c r="A61" s="72" t="s">
         <v>473</v>
@@ -59460,9 +59460,9 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4FAD8CF-47DB-47BD-A145-F803D3707015}">
   <dimension ref="A1:CX43"/>
-  <sheetFormatPr defaultRowHeight="14.3"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="33.625" customWidth="1"/>
+    <col min="1" max="1" width="33.6640625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:102">

</xml_diff>